<commit_message>
cleaned run scripts with hmc/gwmcmc switch, updated readme and plotting
</commit_message>
<xml_diff>
--- a/data/WCdata_RFO.xlsx
+++ b/data/WCdata_RFO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amsuni-my.sharepoint.com/personal/r_f_ott_uva_nl/Documents/Richard/PhD_ETH/matlab/14C_10Be_landscape_transience-master/My_10Be14C_codes/MCMC_inversion/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="8_{83DF1B2F-B15C-49C9-9C7A-A559AC6D8709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42AB5AD1-E939-4B1C-9A39-D720CD928F29}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{83DF1B2F-B15C-49C9-9C7A-A559AC6D8709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9BC42F8-BDC8-464A-A2A3-90F0EB774878}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-18120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -476,6 +476,7 @@
     <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.6640625" customWidth="1"/>
     <col min="6" max="6" width="13.33203125" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
@@ -673,7 +674,7 @@
         <v>49865</v>
       </c>
       <c r="J6">
-        <v>973.82259999999997</v>
+        <v>3809</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -705,7 +706,7 @@
         <v>34375</v>
       </c>
       <c r="J7" s="1">
-        <v>1311.5</v>
+        <v>3658</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
removed GWMCMC and organized repo
</commit_message>
<xml_diff>
--- a/data/WCdata_RFO.xlsx
+++ b/data/WCdata_RFO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amsuni-my.sharepoint.com/personal/r_f_ott_uva_nl/Documents/Richard/PhD_ETH/matlab/14C_10Be_landscape_transience-master/My_10Be14C_codes/MCMC_inversion/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{83DF1B2F-B15C-49C9-9C7A-A559AC6D8709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9BC42F8-BDC8-464A-A2A3-90F0EB774878}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="8_{83DF1B2F-B15C-49C9-9C7A-A559AC6D8709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0968868C-684F-49C5-980D-3DF2F7FCE14C}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-18120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-3060" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
   <si>
     <t>Lat</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t>N26sigma</t>
+  </si>
+  <si>
+    <t>WC-616-16'</t>
   </si>
 </sst>
 </file>
@@ -173,9 +176,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="15">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -205,6 +209,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -470,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
@@ -837,6 +845,38 @@
         <v>2595</v>
       </c>
     </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12">
+        <v>35.163499999999999</v>
+      </c>
+      <c r="C12">
+        <v>24.4742</v>
+      </c>
+      <c r="D12">
+        <v>29000</v>
+      </c>
+      <c r="E12">
+        <v>4300</v>
+      </c>
+      <c r="F12" t="s">
+        <v>2</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>2.65</v>
+      </c>
+      <c r="I12">
+        <v>87594.087128386731</v>
+      </c>
+      <c r="J12">
+        <v>3221.9069332170125</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>

</xml_diff>